<commit_message>
Acrescenta o seguro (970 EUR/ano) aos custos fixos
- Nova seccao de custos anuais na Config, com o seguro a 970 EUR/ano
- O valor mensal do seguro passa a ser calculado (970/12 = 80,83 EUR),
  em vez de escrito a mao
- Linha livre para outros custos anuais (IUC, inspecao, licencas),
  tambem mensalizada automaticamente
- Total de custos fixos mensais: 470,83 EUR

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BoLnRZnZGG2rqos9WDRwrL
</commit_message>
<xml_diff>
--- a/Controlo_TVDE_Lisboa.xlsx
+++ b/Controlo_TVDE_Lisboa.xlsx
@@ -134,30 +134,8 @@
 </comments>
 </file>
 
-<file path=xl/comments7.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <authors>
-    <author>Unknown Author</author>
-  </authors>
-  <commentList>
-    <comment ref="B13" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Valor por preencher. Enquanto estiver vazio conta como 0 € e o resultado mensal aparece melhor do que é na realidade.</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="177">
   <si>
     <t xml:space="preserve">Controlo TVDE — Lisboa</t>
   </si>
@@ -621,28 +599,43 @@
     <t xml:space="preserve">Prestação mensal do Tesla.</t>
   </si>
   <si>
-    <t xml:space="preserve">Seguro</t>
+    <t xml:space="preserve">Seguro (970 €/ano ÷ 12)</t>
   </si>
   <si>
-    <t xml:space="preserve">A PREENCHER — seguro com cobertura de atividade TVDE. Mete o valor mensal assim que o tiveres.</t>
+    <t xml:space="preserve">Calculado a partir do valor anual do seguro, na secção «Custos anuais» abaixo. Muda lá o valor e este acompanha.</t>
   </si>
   <si>
     <t xml:space="preserve">Outros custos fixos 1</t>
   </si>
   <si>
-    <t xml:space="preserve">Livre. Ex.: contabilidade, licenças TVDE mensalizadas, telemóvel, IUC e inspeção divididos por 12.</t>
+    <t xml:space="preserve">Livre, para um custo que pagues TODOS OS MESES. Ex.: contabilidade, telemóvel.</t>
   </si>
   <si>
-    <t xml:space="preserve">Outros custos fixos 2</t>
+    <t xml:space="preserve">Outros custos anuais ÷ 12</t>
   </si>
   <si>
-    <t xml:space="preserve">Livre.</t>
+    <t xml:space="preserve">Calculado a partir do valor anual da secção abaixo. Ex.: IUC, inspeção, licenças TVDE.</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL de custos fixos mensais</t>
   </si>
   <si>
     <t xml:space="preserve">Só entram aqui os custos que listares acima. O que pagares e não estiver nesta lista não é abatido em lado nenhum — o resultado mensal sai por isso melhor do que a realidade.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Custos anuais (entram mensalizados na tabela acima)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seguro (anual)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seguro com cobertura de atividade TVDE. 970 €/ano = 80,83 €/mês, já refletido na tabela acima.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outros custos anuais</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Soma aqui o que pagas uma vez por ano: IUC, inspeção, certificado de motorista TVDE, dístico do veículo.</t>
   </si>
   <si>
     <t xml:space="preserve">Primeiro mês de atividade</t>
@@ -24037,7 +24030,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="43" t="n">
-        <f aca="false">EOMONTH(Config!$B$18,0)</f>
+        <f aca="false">EOMONTH(Config!$B$22,0)</f>
         <v>46295</v>
       </c>
       <c r="B5" s="34" t="n">
@@ -24058,15 +24051,15 @@
       </c>
       <c r="F5" s="44" t="n">
         <f aca="false">IF($B5=0,0,Config!$B$16)</f>
-        <v>390</v>
+        <v>470.833333333333</v>
       </c>
       <c r="G5" s="37" t="n">
         <f aca="false">$E5-$F5</f>
-        <v>-277.86</v>
+        <v>-358.693333333333</v>
       </c>
       <c r="H5" s="37" t="n">
         <f aca="false">IF($C5=0,"",$G5/$C5)</f>
-        <v>-42.7476923076923</v>
+        <v>-55.1835897435897</v>
       </c>
       <c r="I5" s="34" t="n">
         <f aca="false">SUMIFS('Registo Diário'!$M$3:$M$403,'Registo Diário'!$C$3:$C$403,$A5)</f>
@@ -24957,15 +24950,15 @@
       </c>
       <c r="F23" s="41" t="n">
         <f aca="false">SUM(F5:F22)</f>
-        <v>390</v>
+        <v>470.833333333333</v>
       </c>
       <c r="G23" s="41" t="n">
         <f aca="false">SUM(G5:G22)</f>
-        <v>-277.86</v>
+        <v>-358.693333333333</v>
       </c>
       <c r="H23" s="41" t="n">
         <f aca="false">IF($C23=0,"",$G23/$C23)</f>
-        <v>-42.7476923076923</v>
+        <v>-55.1835897435897</v>
       </c>
       <c r="I23" s="39" t="n">
         <f aca="false">SUM(I5:I22)</f>
@@ -25022,7 +25015,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
@@ -25204,7 +25197,10 @@
       <c r="A13" s="33" t="s">
         <v>154</v>
       </c>
-      <c r="B13" s="52"/>
+      <c r="B13" s="30" t="n">
+        <f aca="false">B19/12</f>
+        <v>80.8333333333333</v>
+      </c>
       <c r="C13" s="51" t="s">
         <v>155</v>
       </c>
@@ -25230,7 +25226,8 @@
       <c r="A15" s="33" t="s">
         <v>158</v>
       </c>
-      <c r="B15" s="52" t="n">
+      <c r="B15" s="30" t="n">
+        <f aca="false">B20/12</f>
         <v>0</v>
       </c>
       <c r="C15" s="51" t="s">
@@ -25246,7 +25243,7 @@
       </c>
       <c r="B16" s="41" t="n">
         <f aca="false">SUM(B12:B15)</f>
-        <v>390</v>
+        <v>470.833333333333</v>
       </c>
       <c r="C16" s="55" t="s">
         <v>161</v>
@@ -25261,63 +25258,92 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="33" t="s">
+      <c r="A18" s="49" t="s">
         <v>162</v>
       </c>
-      <c r="B18" s="56" t="n">
+      <c r="B18" s="49"/>
+      <c r="C18" s="49"/>
+    </row>
+    <row r="19" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="33" t="s">
+        <v>163</v>
+      </c>
+      <c r="B19" s="52" t="n">
+        <v>970</v>
+      </c>
+      <c r="C19" s="51" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="33" t="s">
+        <v>165</v>
+      </c>
+      <c r="B20" s="52" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="51" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="33" t="s">
+        <v>167</v>
+      </c>
+      <c r="B22" s="56" t="n">
         <v>46266</v>
       </c>
-      <c r="C18" s="51" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D19" s="46" t="s">
-        <v>164</v>
-      </c>
-      <c r="E19" s="46"/>
-      <c r="F19" s="46"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="49" t="s">
-        <v>165</v>
-      </c>
-      <c r="B20" s="49"/>
-      <c r="C20" s="49"/>
-      <c r="D20" s="46"/>
-      <c r="E20" s="46"/>
-      <c r="F20" s="46"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="57" t="s">
-        <v>166</v>
-      </c>
-      <c r="C21" s="58" t="s">
-        <v>167</v>
-      </c>
-      <c r="D21" s="46"/>
-      <c r="E21" s="46"/>
-      <c r="F21" s="46"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="59" t="s">
+      <c r="C22" s="51" t="s">
         <v>168</v>
       </c>
-      <c r="C22" s="58" t="s">
+      <c r="D22" s="46" t="s">
         <v>169</v>
       </c>
+      <c r="E22" s="46"/>
+      <c r="F22" s="46"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="60" t="s">
+      <c r="D23" s="46"/>
+      <c r="E23" s="46"/>
+      <c r="F23" s="46"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="49" t="s">
         <v>170</v>
       </c>
-      <c r="C23" s="58" t="s">
+      <c r="B24" s="49"/>
+      <c r="C24" s="49"/>
+      <c r="D24" s="46"/>
+      <c r="E24" s="46"/>
+      <c r="F24" s="46"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="57" t="s">
         <v>171</v>
+      </c>
+      <c r="C25" s="58" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="59" t="s">
+        <v>173</v>
+      </c>
+      <c r="C26" s="58" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="60" t="s">
+        <v>175</v>
+      </c>
+      <c r="C27" s="58" t="s">
+        <v>176</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="D19:F21"/>
+    <mergeCell ref="D22:F24"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -25326,6 +25352,5 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>